<commit_message>
Add SEC EDGAR data provider for official financial data retrieval
Co-authored-by: charitos.charitou <charitos.charitou@selwoodam.com>
</commit_message>
<xml_diff>
--- a/fin_analyst_agent/reports/AAPL_DCF.xlsx
+++ b/fin_analyst_agent/reports/AAPL_DCF.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>Assumption</t>
   </si>
@@ -27,6 +27,9 @@
     <t>Ticker</t>
   </si>
   <si>
+    <t>Data Source</t>
+  </si>
+  <si>
     <t>Starting FCF</t>
   </si>
   <si>
@@ -58,6 +61,9 @@
   </si>
   <si>
     <t>AAPL</t>
+  </si>
+  <si>
+    <t>sec</t>
   </si>
   <si>
     <t>Year</t>
@@ -439,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -455,15 +461,15 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>1000000000</v>
+      <c r="B3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -471,7 +477,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>1000000000</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -479,7 +485,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0.05</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -487,7 +493,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -495,7 +501,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -503,7 +509,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -511,7 +517,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.21</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -519,7 +525,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>0.09242500000000001</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -527,7 +533,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.02</v>
+        <v>0.09242500000000001</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -535,6 +541,14 @@
         <v>12</v>
       </c>
       <c r="B12">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
         <v>14840399872</v>
       </c>
     </row>
@@ -550,13 +564,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -626,7 +640,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -634,7 +648,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>4156548423102.162</v>
@@ -642,7 +656,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3">
         <v>2671620040534.036</v>
@@ -650,7 +664,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>2962039872550.265</v>
@@ -658,7 +672,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>199.5929960175042</v>

</xml_diff>